<commit_message>
added reverse engineering for water atomizer
</commit_message>
<xml_diff>
--- a/sw/src/MSPM0_Pins_AssignmentsLab7.xlsx
+++ b/sw/src/MSPM0_Pins_AssignmentsLab7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghakk\ece445l_lab7-10_fall26-4-ew-js-tp-ak\sw\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{223E2441-0589-4651-9B83-F68C468B083D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071FD2E4-C11F-4AB9-A625-5AE9B0CA35B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="866" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="417">
   <si>
     <t>PA25</t>
   </si>
@@ -1187,9 +1187,6 @@
     <t>uC - SPI0_PICO</t>
   </si>
   <si>
-    <t>Free Pins: 2</t>
-  </si>
-  <si>
     <t>Keypad Output 1</t>
   </si>
   <si>
@@ -1220,12 +1217,6 @@
     <t>LEDs</t>
   </si>
   <si>
-    <t>Free Pins: 3</t>
-  </si>
-  <si>
-    <t>(5 if including PA0/1)</t>
-  </si>
-  <si>
     <t>NC</t>
   </si>
   <si>
@@ -1233,6 +1224,96 @@
   </si>
   <si>
     <t>GND</t>
+  </si>
+  <si>
+    <t>ESP8266 Reset</t>
+  </si>
+  <si>
+    <t>ESP8266 GPIO2</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Free Pins: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0</t>
+    </r>
+  </si>
+  <si>
+    <t>Smoke Enable</t>
+  </si>
+  <si>
+    <t>(4 if including PA0/1)</t>
+  </si>
+  <si>
+    <t>Key:</t>
+  </si>
+  <si>
+    <t>Keypad</t>
+  </si>
+  <si>
+    <t>Screen</t>
+  </si>
+  <si>
+    <t>SPI - uC</t>
+  </si>
+  <si>
+    <t>Electromech</t>
+  </si>
+  <si>
+    <t>Speaker</t>
+  </si>
+  <si>
+    <t>Wifi Module</t>
+  </si>
+  <si>
+    <t>ID Reader</t>
+  </si>
+  <si>
+    <t>Flash</t>
+  </si>
+  <si>
+    <t>80MHz SiO2</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Power</t>
+  </si>
+  <si>
+    <t>Unused</t>
+  </si>
+  <si>
+    <t>NC/Free</t>
+  </si>
+  <si>
+    <t>Free</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Free Pins: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3</t>
+    </r>
+  </si>
+  <si>
+    <t>S</t>
   </si>
 </sst>
 </file>
@@ -1242,7 +1323,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1273,8 +1354,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1308,6 +1403,72 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF7C80"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF99CCFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCCFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCCC00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9999FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF99FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1404,7 +1565,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1503,8 +1664,83 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1514,16 +1750,16 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF99FF"/>
+      <color rgb="FF9999FF"/>
+      <color rgb="FFFFFFCC"/>
+      <color rgb="FFCCCC00"/>
+      <color rgb="FFCCFFFF"/>
+      <color rgb="FFCCFFCC"/>
       <color rgb="FF99CCFF"/>
+      <color rgb="FFFFCCFF"/>
       <color rgb="FFFF7C80"/>
-      <color rgb="FFCCFFFF"/>
-      <color rgb="FFFFCCFF"/>
-      <color rgb="FFCCCC00"/>
-      <color rgb="FFFFFFCC"/>
       <color rgb="FFDDDDDD"/>
-      <color rgb="FF9999FF"/>
-      <color rgb="FFFF99FF"/>
-      <color rgb="FFCCFFCC"/>
     </mruColors>
   </colors>
   <extLst>
@@ -5501,15 +5737,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>400050</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>58964</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>419862</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>151738</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>210312</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>29273</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5532,8 +5768,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7231380" y="182880"/>
-          <a:ext cx="7125462" cy="5089498"/>
+          <a:off x="7902121" y="240393"/>
+          <a:ext cx="7103691" cy="5050309"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -12588,7 +12824,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AC81E62-902F-426A-8169-496CDAF34664}">
-  <dimension ref="A1:XEU44"/>
+  <dimension ref="A1:XEU49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.54296875" customWidth="1"/>
@@ -12599,6 +12835,7 @@
     <col min="6" max="6" width="9.08984375" style="2" customWidth="1"/>
     <col min="7" max="7" width="30.36328125" customWidth="1"/>
     <col min="8" max="8" width="5.90625" customWidth="1"/>
+    <col min="9" max="9" width="10.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
@@ -12612,12 +12849,15 @@
         <v>91</v>
       </c>
       <c r="G1" s="7"/>
+      <c r="I1" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" s="11" t="s">
-        <v>390</v>
-      </c>
-      <c r="B2" s="12" t="s">
+      <c r="A2" s="44" t="s">
+        <v>389</v>
+      </c>
+      <c r="B2" s="39" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="18">
@@ -12628,16 +12868,21 @@
         <f t="shared" ref="E2:E15" si="0">E3+1</f>
         <v>32</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="23"/>
+      <c r="G2" s="59" t="s">
+        <v>395</v>
+      </c>
+      <c r="I2" s="43" t="s">
+        <v>401</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="47" t="s">
         <v>210</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="39" t="s">
         <v>15</v>
       </c>
       <c r="C3" s="3">
@@ -12647,16 +12892,19 @@
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="23" t="s">
+      <c r="G3" s="48" t="s">
         <v>213</v>
       </c>
+      <c r="I3" s="46" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="1"/>
-      <c r="B4" s="2" t="s">
+      <c r="A4" s="72"/>
+      <c r="B4" s="39" t="s">
         <v>171</v>
       </c>
       <c r="C4" s="3">
@@ -12666,18 +12914,21 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="G4" t="s">
-        <v>388</v>
+      <c r="G4" s="43" t="s">
+        <v>387</v>
+      </c>
+      <c r="I4" s="51" t="s">
+        <v>403</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>383</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="A5" s="44" t="s">
+        <v>382</v>
+      </c>
+      <c r="B5" s="39" t="s">
         <v>37</v>
       </c>
       <c r="C5" s="3">
@@ -12687,18 +12938,21 @@
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="27" t="s">
+      <c r="G5" s="58" t="s">
         <v>376</v>
       </c>
+      <c r="I5" s="55" t="s">
+        <v>404</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="A6" s="44" t="s">
+        <v>383</v>
+      </c>
+      <c r="B6" s="39" t="s">
         <v>38</v>
       </c>
       <c r="C6" s="3">
@@ -12708,18 +12962,21 @@
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="57" t="s">
         <v>377</v>
       </c>
+      <c r="I6" s="56" t="s">
+        <v>405</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="A7" s="62" t="s">
+        <v>392</v>
+      </c>
+      <c r="B7" s="39" t="s">
         <v>172</v>
       </c>
       <c r="C7" s="3">
@@ -12729,18 +12986,21 @@
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="39" t="s">
         <v>157</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="64" t="s">
         <v>158</v>
       </c>
+      <c r="I7" s="57" t="s">
+        <v>406</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A8" s="38" t="s">
-        <v>396</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="A8" s="71" t="s">
+        <v>393</v>
+      </c>
+      <c r="B8" s="39" t="s">
         <v>173</v>
       </c>
       <c r="C8" s="3">
@@ -12750,18 +13010,21 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="39" t="s">
         <v>155</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="65" t="s">
         <v>156</v>
       </c>
+      <c r="I8" s="63" t="s">
+        <v>407</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>397</v>
-      </c>
-      <c r="B9" s="2" t="s">
+      <c r="A9" s="72" t="s">
+        <v>394</v>
+      </c>
+      <c r="B9" s="39" t="s">
         <v>174</v>
       </c>
       <c r="C9" s="3">
@@ -12771,18 +13034,21 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="F9" s="24" t="s">
+      <c r="F9" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="25" t="s">
+      <c r="G9" s="49" t="s">
         <v>209</v>
       </c>
+      <c r="I9" s="64" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="50" t="s">
         <v>372</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="39" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="3">
@@ -12792,18 +13058,21 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="F10" s="24" t="s">
+      <c r="F10" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="G10" s="25" t="s">
+      <c r="G10" s="49" t="s">
         <v>208</v>
       </c>
+      <c r="I10" s="66" t="s">
+        <v>409</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>385</v>
-      </c>
-      <c r="B11" s="2" t="s">
+      <c r="A11" s="44" t="s">
+        <v>384</v>
+      </c>
+      <c r="B11" s="39" t="s">
         <v>10</v>
       </c>
       <c r="C11" s="3">
@@ -12813,18 +13082,21 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="F11" s="24" t="s">
+      <c r="F11" s="39" t="s">
         <v>153</v>
       </c>
-      <c r="G11" s="25" t="s">
-        <v>207</v>
+      <c r="G11" s="58" t="s">
+        <v>396</v>
+      </c>
+      <c r="I11" s="68" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
-        <v>386</v>
-      </c>
-      <c r="B12" s="2" t="s">
+      <c r="A12" s="44" t="s">
+        <v>385</v>
+      </c>
+      <c r="B12" s="39" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="3">
@@ -12834,18 +13106,21 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="F12" s="16" t="s">
+      <c r="F12" s="39" t="s">
         <v>24</v>
       </c>
       <c r="G12" s="28" t="s">
         <v>362</v>
       </c>
+      <c r="I12" s="61" t="s">
+        <v>413</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="67" t="s">
         <v>176</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="39" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="3">
@@ -12855,18 +13130,21 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="51" t="s">
         <v>373</v>
       </c>
+      <c r="I13" s="70" t="s">
+        <v>411</v>
+      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="67" t="s">
         <v>175</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="39" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="3">
@@ -12876,18 +13154,21 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="F14" s="24" t="s">
+      <c r="F14" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="G14" s="25" t="s">
+      <c r="G14" s="49" t="s">
         <v>212</v>
       </c>
+      <c r="I14" t="s">
+        <v>412</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
-        <v>387</v>
-      </c>
-      <c r="B15" s="2" t="s">
+      <c r="A15" s="44" t="s">
+        <v>386</v>
+      </c>
+      <c r="B15" s="39" t="s">
         <v>14</v>
       </c>
       <c r="C15" s="3">
@@ -12897,10 +13178,10 @@
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="F15" s="13" t="s">
+      <c r="F15" s="39" t="s">
         <v>55</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="51" t="s">
         <v>374</v>
       </c>
       <c r="I15" s="7"/>
@@ -12908,10 +13189,10 @@
       <c r="K15" s="7"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="60" t="s">
         <v>378</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="39" t="s">
         <v>1</v>
       </c>
       <c r="C16" s="3">
@@ -12921,21 +13202,21 @@
         <f>E17+1</f>
         <v>18</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="G16" s="7" t="s">
-        <v>389</v>
+      <c r="G16" s="45" t="s">
+        <v>388</v>
       </c>
       <c r="I16" s="7"/>
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
     </row>
     <row r="17" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="60" t="s">
         <v>379</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="39" t="s">
         <v>88</v>
       </c>
       <c r="C17" s="5">
@@ -12945,10 +13226,10 @@
       <c r="E17" s="6">
         <v>17</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="G17" s="52" t="s">
         <v>375</v>
       </c>
       <c r="I17" s="7"/>
@@ -12956,33 +13237,38 @@
       <c r="K17" s="7"/>
     </row>
     <row r="18" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A18" s="1" t="s">
-        <v>382</v>
-      </c>
+      <c r="A18" s="38" t="s">
+        <v>397</v>
+      </c>
+      <c r="B18" s="38"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="40"/>
       <c r="I18" s="7"/>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
     </row>
     <row r="19" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+      <c r="A19" s="40" t="s">
         <v>370</v>
       </c>
+      <c r="B19" s="38"/>
       <c r="C19" s="2" t="s">
         <v>91</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="G19" s="7"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="42"/>
       <c r="I19" s="7"/>
       <c r="J19" s="7"/>
       <c r="K19" s="7"/>
     </row>
     <row r="20" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="53" t="s">
         <v>365</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="39" t="s">
         <v>3</v>
       </c>
       <c r="C20" s="18">
@@ -12993,10 +13279,10 @@
         <f t="shared" ref="E20:E33" si="1">E21+1</f>
         <v>32</v>
       </c>
-      <c r="F20" s="22" t="s">
+      <c r="F20" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="G20" s="23" t="s">
+      <c r="G20" s="48" t="s">
         <v>211</v>
       </c>
       <c r="I20" s="7"/>
@@ -13004,10 +13290,10 @@
       <c r="K20" s="7"/>
     </row>
     <row r="21" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="47" t="s">
         <v>210</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="39" t="s">
         <v>15</v>
       </c>
       <c r="C21" s="3">
@@ -13017,10 +13303,10 @@
         <f t="shared" si="1"/>
         <v>31</v>
       </c>
-      <c r="F21" s="22" t="s">
+      <c r="F21" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="G21" s="23" t="s">
+      <c r="G21" s="48" t="s">
         <v>213</v>
       </c>
       <c r="I21" s="7"/>
@@ -13028,8 +13314,8 @@
       <c r="K21" s="7"/>
     </row>
     <row r="22" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A22" s="1"/>
-      <c r="B22" s="2" t="s">
+      <c r="A22" s="72"/>
+      <c r="B22" s="39" t="s">
         <v>171</v>
       </c>
       <c r="C22" s="3">
@@ -13039,10 +13325,10 @@
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F22" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="G22" s="26" t="s">
+      <c r="G22" s="54" t="s">
         <v>366</v>
       </c>
       <c r="I22" s="7"/>
@@ -13050,10 +13336,10 @@
       <c r="K22" s="7"/>
     </row>
     <row r="23" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="B23" s="2" t="s">
+      <c r="A23" s="62" t="s">
+        <v>392</v>
+      </c>
+      <c r="B23" s="39" t="s">
         <v>37</v>
       </c>
       <c r="C23" s="3">
@@ -13063,21 +13349,21 @@
         <f t="shared" si="1"/>
         <v>29</v>
       </c>
-      <c r="F23" s="17" t="s">
+      <c r="F23" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="G23" t="s">
-        <v>391</v>
+      <c r="G23" s="55" t="s">
+        <v>390</v>
       </c>
       <c r="I23" s="7"/>
       <c r="J23" s="7"/>
       <c r="K23" s="7"/>
     </row>
     <row r="24" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="B24" s="2" t="s">
+      <c r="A24" s="69" t="s">
+        <v>398</v>
+      </c>
+      <c r="B24" s="39" t="s">
         <v>38</v>
       </c>
       <c r="C24" s="3">
@@ -13087,21 +13373,21 @@
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="G24" t="s">
-        <v>392</v>
+      <c r="G24" s="68" t="s">
+        <v>391</v>
       </c>
       <c r="I24" s="7"/>
       <c r="J24" s="7"/>
       <c r="K24" s="7"/>
     </row>
     <row r="25" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="B25" s="2" t="s">
+      <c r="A25" s="62" t="s">
+        <v>392</v>
+      </c>
+      <c r="B25" s="39" t="s">
         <v>172</v>
       </c>
       <c r="C25" s="3">
@@ -13111,10 +13397,10 @@
         <f t="shared" si="1"/>
         <v>27</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F25" s="39" t="s">
         <v>157</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="64" t="s">
         <v>158</v>
       </c>
       <c r="I25" s="7"/>
@@ -13122,10 +13408,10 @@
       <c r="K25" s="7"/>
     </row>
     <row r="26" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A26" s="38" t="s">
-        <v>396</v>
-      </c>
-      <c r="B26" s="2" t="s">
+      <c r="A26" s="71" t="s">
+        <v>393</v>
+      </c>
+      <c r="B26" s="39" t="s">
         <v>173</v>
       </c>
       <c r="C26" s="3">
@@ -13135,10 +13421,10 @@
         <f t="shared" si="1"/>
         <v>26</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" s="39" t="s">
         <v>155</v>
       </c>
-      <c r="G26" s="7" t="s">
+      <c r="G26" s="65" t="s">
         <v>156</v>
       </c>
       <c r="I26" s="7"/>
@@ -13146,10 +13432,10 @@
       <c r="K26" s="7"/>
     </row>
     <row r="27" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
-        <v>397</v>
-      </c>
-      <c r="B27" s="2" t="s">
+      <c r="A27" s="72" t="s">
+        <v>394</v>
+      </c>
+      <c r="B27" s="39" t="s">
         <v>174</v>
       </c>
       <c r="C27" s="3">
@@ -13159,10 +13445,10 @@
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="F27" s="24" t="s">
+      <c r="F27" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="G27" s="25" t="s">
+      <c r="G27" s="49" t="s">
         <v>209</v>
       </c>
       <c r="I27" s="7"/>
@@ -13170,10 +13456,10 @@
       <c r="K27" s="7"/>
     </row>
     <row r="28" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
+      <c r="A28" s="50" t="s">
         <v>372</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="39" t="s">
         <v>9</v>
       </c>
       <c r="C28" s="3">
@@ -13183,10 +13469,10 @@
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="F28" s="24" t="s">
+      <c r="F28" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="G28" s="25" t="s">
+      <c r="G28" s="49" t="s">
         <v>208</v>
       </c>
       <c r="I28" s="7"/>
@@ -13194,8 +13480,10 @@
       <c r="K28" s="7"/>
     </row>
     <row r="29" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A29" s="1"/>
-      <c r="B29" s="2" t="s">
+      <c r="A29" s="62" t="s">
+        <v>414</v>
+      </c>
+      <c r="B29" s="39" t="s">
         <v>10</v>
       </c>
       <c r="C29" s="3">
@@ -13205,19 +13493,19 @@
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
-      <c r="F29" s="24" t="s">
+      <c r="F29" s="39" t="s">
         <v>153</v>
       </c>
-      <c r="G29" s="25" t="s">
+      <c r="G29" s="49" t="s">
         <v>207</v>
       </c>
       <c r="K29" s="7"/>
     </row>
     <row r="30" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A30" s="1" t="s">
+      <c r="A30" s="50" t="s">
         <v>380</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="39" t="s">
         <v>11</v>
       </c>
       <c r="C30" s="3">
@@ -13227,7 +13515,7 @@
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="F30" s="16" t="s">
+      <c r="F30" s="39" t="s">
         <v>24</v>
       </c>
       <c r="G30" s="28" t="s">
@@ -13237,10 +13525,10 @@
       <c r="J30" s="7"/>
     </row>
     <row r="31" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="67" t="s">
         <v>176</v>
       </c>
-      <c r="B31" s="12" t="s">
+      <c r="B31" s="39" t="s">
         <v>12</v>
       </c>
       <c r="C31" s="3">
@@ -13250,8 +13538,11 @@
         <f t="shared" si="1"/>
         <v>21</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="F31" s="39" t="s">
         <v>39</v>
+      </c>
+      <c r="G31" s="73" t="s">
+        <v>414</v>
       </c>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
@@ -19393,10 +19684,10 @@
       <c r="XEU31" s="2"/>
     </row>
     <row r="32" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="67" t="s">
         <v>175</v>
       </c>
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="39" t="s">
         <v>13</v>
       </c>
       <c r="C32" s="3">
@@ -19406,16 +19697,18 @@
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="F32" s="24" t="s">
+      <c r="F32" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="G32" s="25" t="s">
+      <c r="G32" s="49" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" s="1"/>
-      <c r="B33" s="2" t="s">
+      <c r="A33" s="62" t="s">
+        <v>414</v>
+      </c>
+      <c r="B33" s="39" t="s">
         <v>14</v>
       </c>
       <c r="C33" s="3">
@@ -19425,18 +19718,18 @@
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
-      <c r="F33" s="13" t="s">
+      <c r="F33" s="39" t="s">
         <v>55</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G33" s="55" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" s="1" t="s">
+      <c r="A34" s="53" t="s">
         <v>367</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="39" t="s">
         <v>1</v>
       </c>
       <c r="C34" s="3">
@@ -19446,18 +19739,18 @@
         <f>E35+1</f>
         <v>18</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="F34" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G34" s="51" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" s="1" t="s">
+      <c r="A35" s="50" t="s">
         <v>381</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="39" t="s">
         <v>88</v>
       </c>
       <c r="C35" s="5">
@@ -19467,22 +19760,22 @@
       <c r="E35" s="6">
         <v>17</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="F35" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="G35" s="7" t="s">
+      <c r="G35" s="54" t="s">
         <v>368</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
-        <v>393</v>
+        <v>415</v>
       </c>
       <c r="B36"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="B37"/>
     </row>
@@ -19516,6 +19809,11 @@
       <c r="C44"/>
       <c r="D44"/>
       <c r="E44"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>416</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
finished prelim layout for TA review
</commit_message>
<xml_diff>
--- a/sw/src/MSPM0_Pins_AssignmentsLab7.xlsx
+++ b/sw/src/MSPM0_Pins_AssignmentsLab7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghakk\ece445l_lab7-10_fall26-4-ew-js-tp-ak\sw\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5557FAB4-C80B-4455-A2E2-56555B9F6CB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0600022-1FFE-4E09-A523-ADF0C02DC7B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,20 @@
     <sheet name="ADC" sheetId="12" r:id="rId6"/>
     <sheet name="PINCM" sheetId="11" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1196,9 +1209,6 @@
   </si>
   <si>
     <t>Keypad Input 4</t>
-  </si>
-  <si>
-    <t>Flywheels</t>
   </si>
   <si>
     <t>NC</t>
@@ -1297,13 +1307,16 @@
     <t>S</t>
   </si>
   <si>
-    <t>LED Group 1</t>
-  </si>
-  <si>
     <t>LED Group 2</t>
   </si>
   <si>
     <t>Motor PWM</t>
+  </si>
+  <si>
+    <t>Winch+</t>
+  </si>
+  <si>
+    <t>Winch-</t>
   </si>
 </sst>
 </file>
@@ -12827,7 +12840,7 @@
       </c>
       <c r="G1" s="7"/>
       <c r="I1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
@@ -12849,10 +12862,10 @@
         <v>0</v>
       </c>
       <c r="G2" s="55" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I2" s="39" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
@@ -12876,7 +12889,7 @@
         <v>213</v>
       </c>
       <c r="I3" s="42" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
@@ -12898,7 +12911,7 @@
         <v>387</v>
       </c>
       <c r="I4" s="47" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
@@ -12922,7 +12935,7 @@
         <v>376</v>
       </c>
       <c r="I5" s="51" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
@@ -12946,12 +12959,12 @@
         <v>377</v>
       </c>
       <c r="I6" s="52" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="58" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>172</v>
@@ -12970,12 +12983,12 @@
         <v>158</v>
       </c>
       <c r="I7" s="53" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="67" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>173</v>
@@ -12994,12 +13007,12 @@
         <v>156</v>
       </c>
       <c r="I8" s="59" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="68" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>174</v>
@@ -13018,7 +13031,7 @@
         <v>209</v>
       </c>
       <c r="I9" s="60" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
@@ -13042,7 +13055,7 @@
         <v>208</v>
       </c>
       <c r="I10" s="62" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
@@ -13063,10 +13076,10 @@
         <v>153</v>
       </c>
       <c r="G11" s="54" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="I11" s="64" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
@@ -13090,7 +13103,7 @@
         <v>362</v>
       </c>
       <c r="I12" s="57" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
@@ -13114,7 +13127,7 @@
         <v>373</v>
       </c>
       <c r="I13" s="66" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
@@ -13138,7 +13151,7 @@
         <v>212</v>
       </c>
       <c r="I14" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
@@ -13215,7 +13228,7 @@
     </row>
     <row r="18" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="I18" s="7"/>
       <c r="J18" s="7"/>
@@ -13309,7 +13322,7 @@
     </row>
     <row r="23" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
       <c r="A23" s="49" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>37</v>
@@ -13325,7 +13338,7 @@
         <v>19</v>
       </c>
       <c r="G23" s="51" t="s">
-        <v>390</v>
+        <v>416</v>
       </c>
       <c r="I23" s="7"/>
       <c r="J23" s="7"/>
@@ -13333,7 +13346,7 @@
     </row>
     <row r="24" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
       <c r="A24" s="65" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>38</v>
@@ -13348,8 +13361,8 @@
       <c r="F24" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="G24" s="64" t="s">
-        <v>415</v>
+      <c r="G24" s="51" t="s">
+        <v>417</v>
       </c>
       <c r="I24" s="7"/>
       <c r="J24" s="7"/>
@@ -13357,7 +13370,7 @@
     </row>
     <row r="25" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
       <c r="A25" s="58" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>172</v>
@@ -13381,7 +13394,7 @@
     </row>
     <row r="26" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
       <c r="A26" s="67" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>173</v>
@@ -13405,7 +13418,7 @@
     </row>
     <row r="27" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
       <c r="A27" s="68" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>174</v>
@@ -13453,7 +13466,7 @@
     </row>
     <row r="29" spans="1:1023 1029:2047 2053:3071 3077:4095 4101:5119 5125:6143 6149:7167 7173:8191 8197:9215 9221:10239 10245:11263 11269:12287 12293:13311 13317:14335 14341:15359 15365:16375" x14ac:dyDescent="0.35">
       <c r="A29" s="58" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>10</v>
@@ -13514,7 +13527,7 @@
         <v>39</v>
       </c>
       <c r="G31" s="64" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
@@ -19678,7 +19691,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="58" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>14</v>
@@ -19741,7 +19754,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B36"/>
     </row>
@@ -19782,7 +19795,7 @@
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
   </sheetData>

</xml_diff>